<commit_message>
fix missing/duplicates in dpv, dpv/legal_basis
See Issue #127

-  dpv_legal_basis: Missing concepts for terms defined in main
   vocabulary e.g. dpv:Context
-  dpv: Resolve multiple contributors in term definition e.g.
   isImplementedByEntity
-  dpv: Resolve multiple creation dates in term definition e.g.
   isImplementedByEntity
</commit_message>
<xml_diff>
--- a/code/vocab_csv/rights.xlsx
+++ b/code/vocab_csv/rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="307">
   <si>
     <t>Term</t>
   </si>
@@ -5780,16 +5780,12 @@
       <c r="H4" s="19"/>
       <c r="I4" s="19"/>
       <c r="J4" s="19"/>
-      <c r="K4" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K4" s="21"/>
       <c r="L4" s="19"/>
       <c r="M4" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N4" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N4" s="19"/>
       <c r="O4" s="33" t="s">
         <v>22</v>
       </c>
@@ -5830,16 +5826,12 @@
       <c r="H5" s="19"/>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K5" s="21"/>
       <c r="L5" s="19"/>
       <c r="M5" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N5" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N5" s="19"/>
       <c r="O5" s="33" t="s">
         <v>22</v>
       </c>
@@ -5880,16 +5872,12 @@
       <c r="H6" s="19"/>
       <c r="I6" s="19"/>
       <c r="J6" s="19"/>
-      <c r="K6" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K6" s="21"/>
       <c r="L6" s="19"/>
       <c r="M6" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N6" s="19"/>
       <c r="O6" s="33" t="s">
         <v>22</v>
       </c>
@@ -5928,16 +5916,12 @@
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
-      <c r="K7" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K7" s="21"/>
       <c r="L7" s="19"/>
       <c r="M7" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N7" s="19"/>
       <c r="O7" s="33" t="s">
         <v>22</v>
       </c>
@@ -5978,16 +5962,12 @@
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
-      <c r="K8" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K8" s="21"/>
       <c r="L8" s="19"/>
       <c r="M8" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N8" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N8" s="19"/>
       <c r="O8" s="33" t="s">
         <v>22</v>
       </c>
@@ -6028,16 +6008,12 @@
       <c r="H9" s="19"/>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
-      <c r="K9" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K9" s="21"/>
       <c r="L9" s="19"/>
       <c r="M9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N9" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N9" s="19"/>
       <c r="O9" s="33" t="s">
         <v>22</v>
       </c>
@@ -6078,16 +6054,12 @@
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
       <c r="J10" s="19"/>
-      <c r="K10" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K10" s="21"/>
       <c r="L10" s="19"/>
       <c r="M10" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N10" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N10" s="19"/>
       <c r="O10" s="33" t="s">
         <v>22</v>
       </c>
@@ -6128,16 +6100,12 @@
       <c r="H11" s="19"/>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
-      <c r="K11" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K11" s="21"/>
       <c r="L11" s="19"/>
       <c r="M11" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N11" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N11" s="19"/>
       <c r="O11" s="33" t="s">
         <v>22</v>
       </c>
@@ -6178,16 +6146,12 @@
       <c r="H12" s="19"/>
       <c r="I12" s="19"/>
       <c r="J12" s="19"/>
-      <c r="K12" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K12" s="21"/>
       <c r="L12" s="19"/>
       <c r="M12" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N12" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N12" s="19"/>
       <c r="O12" s="33" t="s">
         <v>22</v>
       </c>
@@ -6224,16 +6188,12 @@
       <c r="H13" s="19"/>
       <c r="I13" s="19"/>
       <c r="J13" s="19"/>
-      <c r="K13" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K13" s="21"/>
       <c r="L13" s="19"/>
       <c r="M13" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N13" s="19"/>
       <c r="O13" s="33" t="s">
         <v>22</v>
       </c>
@@ -6270,16 +6230,12 @@
       <c r="H14" s="19"/>
       <c r="I14" s="19"/>
       <c r="J14" s="19"/>
-      <c r="K14" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K14" s="21"/>
       <c r="L14" s="19"/>
       <c r="M14" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N14" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N14" s="19"/>
       <c r="O14" s="33" t="s">
         <v>22</v>
       </c>
@@ -6316,16 +6272,12 @@
       <c r="H15" s="19"/>
       <c r="I15" s="19"/>
       <c r="J15" s="19"/>
-      <c r="K15" s="21">
-        <v>44867.0</v>
-      </c>
+      <c r="K15" s="21"/>
       <c r="L15" s="19"/>
       <c r="M15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="N15" s="18" t="s">
-        <v>75</v>
-      </c>
+      <c r="N15" s="19"/>
       <c r="O15" s="33" t="s">
         <v>22</v>
       </c>

</xml_diff>